<commit_message>
Excel Arreglado GUI 04
</commit_message>
<xml_diff>
--- a/ProyectoAsistencia/ReporteClasesDeLaboratorio.xlsx
+++ b/ProyectoAsistencia/ReporteClasesDeLaboratorio.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="177">
   <si>
     <t>Nro Laboratorio</t>
   </si>
@@ -41,6 +41,27 @@
     <t>LAB-101</t>
   </si>
   <si>
+    <t>Matemáticas I</t>
+  </si>
+  <si>
+    <t>juanperez</t>
+  </si>
+  <si>
+    <t>LUNES</t>
+  </si>
+  <si>
+    <t>08:00:00</t>
+  </si>
+  <si>
+    <t>10:00:00</t>
+  </si>
+  <si>
+    <t>02-12-2024</t>
+  </si>
+  <si>
+    <t>HS01</t>
+  </si>
+  <si>
     <t>Estructuras Discretas</t>
   </si>
   <si>
@@ -50,12 +71,6 @@
     <t>MARTES</t>
   </si>
   <si>
-    <t>08:00:00</t>
-  </si>
-  <si>
-    <t>10:00:00</t>
-  </si>
-  <si>
     <t>08-12-2024</t>
   </si>
   <si>
@@ -107,6 +122,18 @@
     <t>HS25</t>
   </si>
   <si>
+    <t>adrianasantos</t>
+  </si>
+  <si>
+    <t>SABADO</t>
+  </si>
+  <si>
+    <t>01-01-2025</t>
+  </si>
+  <si>
+    <t>HS31</t>
+  </si>
+  <si>
     <t>doloresjimenez</t>
   </si>
   <si>
@@ -128,9 +155,6 @@
     <t>anagonzalez</t>
   </si>
   <si>
-    <t>LUNES</t>
-  </si>
-  <si>
     <t>12:00:00</t>
   </si>
   <si>
@@ -191,9 +215,6 @@
     <t>tomasgutierrez</t>
   </si>
   <si>
-    <t>SABADO</t>
-  </si>
-  <si>
     <t>02-01-2025</t>
   </si>
   <si>
@@ -431,6 +452,18 @@
     <t>HS23</t>
   </si>
   <si>
+    <t>Ética Profesional</t>
+  </si>
+  <si>
+    <t>rosacastro</t>
+  </si>
+  <si>
+    <t>30-12-2024</t>
+  </si>
+  <si>
+    <t>HS29</t>
+  </si>
+  <si>
     <t>luisanaponce</t>
   </si>
   <si>
@@ -489,6 +522,18 @@
   </si>
   <si>
     <t>HS24</t>
+  </si>
+  <si>
+    <t>Economía y Gestión de la Tecnología</t>
+  </si>
+  <si>
+    <t>victorsalazar</t>
+  </si>
+  <si>
+    <t>31-12-2024</t>
+  </si>
+  <si>
+    <t>HS30</t>
   </si>
   <si>
     <t>estebanherrera</t>
@@ -542,7 +587,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:I41"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="25.0" customWidth="true"/>
@@ -690,13 +735,13 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>9</v>
+        <v>31</v>
       </c>
       <c r="C6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E6" t="s">
         <v>12</v>
@@ -705,82 +750,82 @@
         <v>13</v>
       </c>
       <c r="G6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>35</v>
+        <v>8</v>
       </c>
       <c r="B7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" t="s">
         <v>36</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>37</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G7" t="s">
         <v>38</v>
       </c>
-      <c r="E7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F7" t="s">
+      <c r="H7" t="s">
         <v>39</v>
-      </c>
-      <c r="G7" t="s">
-        <v>40</v>
-      </c>
-      <c r="H7" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>35</v>
+        <v>8</v>
       </c>
       <c r="B8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" t="s">
+        <v>40</v>
+      </c>
+      <c r="D8" t="s">
+        <v>41</v>
+      </c>
+      <c r="E8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" t="s">
+        <v>13</v>
+      </c>
+      <c r="G8" t="s">
         <v>42</v>
       </c>
-      <c r="C8" t="s">
+      <c r="H8" t="s">
         <v>43</v>
-      </c>
-      <c r="D8" t="s">
-        <v>11</v>
-      </c>
-      <c r="E8" t="s">
-        <v>13</v>
-      </c>
-      <c r="F8" t="s">
-        <v>39</v>
-      </c>
-      <c r="G8" t="s">
-        <v>44</v>
-      </c>
-      <c r="H8" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="B9" t="s">
+        <v>45</v>
+      </c>
+      <c r="C9" t="s">
         <v>46</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" t="s">
         <v>47</v>
-      </c>
-      <c r="D9" t="s">
-        <v>18</v>
-      </c>
-      <c r="E9" t="s">
-        <v>13</v>
-      </c>
-      <c r="F9" t="s">
-        <v>39</v>
       </c>
       <c r="G9" t="s">
         <v>48</v>
@@ -791,7 +836,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="B10" t="s">
         <v>50</v>
@@ -800,13 +845,13 @@
         <v>51</v>
       </c>
       <c r="D10" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="E10" t="s">
         <v>13</v>
       </c>
       <c r="F10" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="G10" t="s">
         <v>52</v>
@@ -817,7 +862,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="B11" t="s">
         <v>54</v>
@@ -826,13 +871,13 @@
         <v>55</v>
       </c>
       <c r="D11" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="E11" t="s">
         <v>13</v>
       </c>
       <c r="F11" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="G11" t="s">
         <v>56</v>
@@ -843,22 +888,22 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="B12" t="s">
-        <v>36</v>
+        <v>58</v>
       </c>
       <c r="C12" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D12" t="s">
-        <v>59</v>
+        <v>28</v>
       </c>
       <c r="E12" t="s">
         <v>13</v>
       </c>
       <c r="F12" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="G12" t="s">
         <v>60</v>
@@ -869,178 +914,178 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="B13" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="C13" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D13" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E13" t="s">
         <v>13</v>
       </c>
       <c r="F13" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="G13" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H13" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>65</v>
+        <v>44</v>
       </c>
       <c r="B14" t="s">
+        <v>45</v>
+      </c>
+      <c r="C14" t="s">
         <v>66</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
+        <v>37</v>
+      </c>
+      <c r="E14" t="s">
+        <v>13</v>
+      </c>
+      <c r="F14" t="s">
+        <v>47</v>
+      </c>
+      <c r="G14" t="s">
         <v>67</v>
       </c>
-      <c r="D14" t="s">
-        <v>38</v>
-      </c>
-      <c r="E14" t="s">
-        <v>39</v>
-      </c>
-      <c r="F14" t="s">
+      <c r="H14" t="s">
         <v>68</v>
-      </c>
-      <c r="G14" t="s">
-        <v>69</v>
-      </c>
-      <c r="H14" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>65</v>
+        <v>44</v>
       </c>
       <c r="B15" t="s">
+        <v>50</v>
+      </c>
+      <c r="C15" t="s">
+        <v>69</v>
+      </c>
+      <c r="D15" t="s">
+        <v>41</v>
+      </c>
+      <c r="E15" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" t="s">
+        <v>47</v>
+      </c>
+      <c r="G15" t="s">
+        <v>70</v>
+      </c>
+      <c r="H15" t="s">
         <v>71</v>
-      </c>
-      <c r="C15" t="s">
-        <v>72</v>
-      </c>
-      <c r="D15" t="s">
-        <v>11</v>
-      </c>
-      <c r="E15" t="s">
-        <v>39</v>
-      </c>
-      <c r="F15" t="s">
-        <v>68</v>
-      </c>
-      <c r="G15" t="s">
-        <v>73</v>
-      </c>
-      <c r="H15" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="B16" t="s">
+        <v>73</v>
+      </c>
+      <c r="C16" t="s">
+        <v>74</v>
+      </c>
+      <c r="D16" t="s">
+        <v>11</v>
+      </c>
+      <c r="E16" t="s">
+        <v>47</v>
+      </c>
+      <c r="F16" t="s">
         <v>75</v>
       </c>
-      <c r="C16" t="s">
+      <c r="G16" t="s">
         <v>76</v>
       </c>
-      <c r="D16" t="s">
-        <v>18</v>
-      </c>
-      <c r="E16" t="s">
-        <v>39</v>
-      </c>
-      <c r="F16" t="s">
-        <v>68</v>
-      </c>
-      <c r="G16" t="s">
+      <c r="H16" t="s">
         <v>77</v>
-      </c>
-      <c r="H16" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="B17" t="s">
+        <v>78</v>
+      </c>
+      <c r="C17" t="s">
         <v>79</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D17" t="s">
+        <v>18</v>
+      </c>
+      <c r="E17" t="s">
+        <v>47</v>
+      </c>
+      <c r="F17" t="s">
+        <v>75</v>
+      </c>
+      <c r="G17" t="s">
         <v>80</v>
       </c>
-      <c r="D17" t="s">
-        <v>23</v>
-      </c>
-      <c r="E17" t="s">
-        <v>39</v>
-      </c>
-      <c r="F17" t="s">
-        <v>68</v>
-      </c>
-      <c r="G17" t="s">
+      <c r="H17" t="s">
         <v>81</v>
-      </c>
-      <c r="H17" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="B18" t="s">
+        <v>82</v>
+      </c>
+      <c r="C18" t="s">
         <v>83</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D18" t="s">
+        <v>23</v>
+      </c>
+      <c r="E18" t="s">
+        <v>47</v>
+      </c>
+      <c r="F18" t="s">
+        <v>75</v>
+      </c>
+      <c r="G18" t="s">
         <v>84</v>
       </c>
-      <c r="D18" t="s">
-        <v>28</v>
-      </c>
-      <c r="E18" t="s">
-        <v>39</v>
-      </c>
-      <c r="F18" t="s">
-        <v>68</v>
-      </c>
-      <c r="G18" t="s">
+      <c r="H18" t="s">
         <v>85</v>
-      </c>
-      <c r="H18" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="B19" t="s">
-        <v>66</v>
+        <v>86</v>
       </c>
       <c r="C19" t="s">
         <v>87</v>
       </c>
       <c r="D19" t="s">
-        <v>59</v>
+        <v>28</v>
       </c>
       <c r="E19" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="F19" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="G19" t="s">
         <v>88</v>
@@ -1051,178 +1096,178 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="B20" t="s">
-        <v>71</v>
+        <v>90</v>
       </c>
       <c r="C20" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D20" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E20" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="F20" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="G20" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="H20" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>93</v>
+        <v>72</v>
       </c>
       <c r="B21" t="s">
+        <v>73</v>
+      </c>
+      <c r="C21" t="s">
         <v>94</v>
       </c>
-      <c r="C21" t="s">
+      <c r="D21" t="s">
+        <v>37</v>
+      </c>
+      <c r="E21" t="s">
+        <v>47</v>
+      </c>
+      <c r="F21" t="s">
+        <v>75</v>
+      </c>
+      <c r="G21" t="s">
         <v>95</v>
       </c>
-      <c r="D21" t="s">
-        <v>38</v>
-      </c>
-      <c r="E21" t="s">
-        <v>68</v>
-      </c>
-      <c r="F21" t="s">
+      <c r="H21" t="s">
         <v>96</v>
-      </c>
-      <c r="G21" t="s">
-        <v>97</v>
-      </c>
-      <c r="H21" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>93</v>
+        <v>72</v>
       </c>
       <c r="B22" t="s">
+        <v>78</v>
+      </c>
+      <c r="C22" t="s">
+        <v>97</v>
+      </c>
+      <c r="D22" t="s">
+        <v>41</v>
+      </c>
+      <c r="E22" t="s">
+        <v>47</v>
+      </c>
+      <c r="F22" t="s">
+        <v>75</v>
+      </c>
+      <c r="G22" t="s">
+        <v>98</v>
+      </c>
+      <c r="H22" t="s">
         <v>99</v>
-      </c>
-      <c r="C22" t="s">
-        <v>100</v>
-      </c>
-      <c r="D22" t="s">
-        <v>11</v>
-      </c>
-      <c r="E22" t="s">
-        <v>68</v>
-      </c>
-      <c r="F22" t="s">
-        <v>96</v>
-      </c>
-      <c r="G22" t="s">
-        <v>101</v>
-      </c>
-      <c r="H22" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="B23" t="s">
+        <v>101</v>
+      </c>
+      <c r="C23" t="s">
+        <v>102</v>
+      </c>
+      <c r="D23" t="s">
+        <v>11</v>
+      </c>
+      <c r="E23" t="s">
+        <v>75</v>
+      </c>
+      <c r="F23" t="s">
         <v>103</v>
       </c>
-      <c r="C23" t="s">
+      <c r="G23" t="s">
         <v>104</v>
       </c>
-      <c r="D23" t="s">
-        <v>18</v>
-      </c>
-      <c r="E23" t="s">
-        <v>68</v>
-      </c>
-      <c r="F23" t="s">
-        <v>96</v>
-      </c>
-      <c r="G23" t="s">
+      <c r="H23" t="s">
         <v>105</v>
-      </c>
-      <c r="H23" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="B24" t="s">
+        <v>106</v>
+      </c>
+      <c r="C24" t="s">
         <v>107</v>
       </c>
-      <c r="C24" t="s">
+      <c r="D24" t="s">
+        <v>18</v>
+      </c>
+      <c r="E24" t="s">
+        <v>75</v>
+      </c>
+      <c r="F24" t="s">
+        <v>103</v>
+      </c>
+      <c r="G24" t="s">
         <v>108</v>
       </c>
-      <c r="D24" t="s">
-        <v>23</v>
-      </c>
-      <c r="E24" t="s">
-        <v>68</v>
-      </c>
-      <c r="F24" t="s">
-        <v>96</v>
-      </c>
-      <c r="G24" t="s">
+      <c r="H24" t="s">
         <v>109</v>
-      </c>
-      <c r="H24" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="B25" t="s">
+        <v>110</v>
+      </c>
+      <c r="C25" t="s">
         <v>111</v>
       </c>
-      <c r="C25" t="s">
+      <c r="D25" t="s">
+        <v>23</v>
+      </c>
+      <c r="E25" t="s">
+        <v>75</v>
+      </c>
+      <c r="F25" t="s">
+        <v>103</v>
+      </c>
+      <c r="G25" t="s">
         <v>112</v>
       </c>
-      <c r="D25" t="s">
-        <v>28</v>
-      </c>
-      <c r="E25" t="s">
-        <v>68</v>
-      </c>
-      <c r="F25" t="s">
-        <v>96</v>
-      </c>
-      <c r="G25" t="s">
+      <c r="H25" t="s">
         <v>113</v>
-      </c>
-      <c r="H25" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="B26" t="s">
-        <v>94</v>
+        <v>114</v>
       </c>
       <c r="C26" t="s">
         <v>115</v>
       </c>
       <c r="D26" t="s">
-        <v>59</v>
+        <v>28</v>
       </c>
       <c r="E26" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="F26" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="G26" t="s">
         <v>116</v>
@@ -1233,152 +1278,152 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="B27" t="s">
-        <v>99</v>
+        <v>118</v>
       </c>
       <c r="C27" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D27" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E27" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="F27" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="G27" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H27" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>121</v>
+        <v>100</v>
       </c>
       <c r="B28" t="s">
+        <v>101</v>
+      </c>
+      <c r="C28" t="s">
         <v>122</v>
       </c>
-      <c r="C28" t="s">
+      <c r="D28" t="s">
+        <v>37</v>
+      </c>
+      <c r="E28" t="s">
+        <v>75</v>
+      </c>
+      <c r="F28" t="s">
+        <v>103</v>
+      </c>
+      <c r="G28" t="s">
         <v>123</v>
       </c>
-      <c r="D28" t="s">
-        <v>38</v>
-      </c>
-      <c r="E28" t="s">
-        <v>96</v>
-      </c>
-      <c r="F28" t="s">
+      <c r="H28" t="s">
         <v>124</v>
-      </c>
-      <c r="G28" t="s">
-        <v>125</v>
-      </c>
-      <c r="H28" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>121</v>
+        <v>100</v>
       </c>
       <c r="B29" t="s">
+        <v>106</v>
+      </c>
+      <c r="C29" t="s">
+        <v>125</v>
+      </c>
+      <c r="D29" t="s">
+        <v>41</v>
+      </c>
+      <c r="E29" t="s">
+        <v>75</v>
+      </c>
+      <c r="F29" t="s">
+        <v>103</v>
+      </c>
+      <c r="G29" t="s">
+        <v>126</v>
+      </c>
+      <c r="H29" t="s">
         <v>127</v>
-      </c>
-      <c r="C29" t="s">
-        <v>128</v>
-      </c>
-      <c r="D29" t="s">
-        <v>11</v>
-      </c>
-      <c r="E29" t="s">
-        <v>96</v>
-      </c>
-      <c r="F29" t="s">
-        <v>124</v>
-      </c>
-      <c r="G29" t="s">
-        <v>129</v>
-      </c>
-      <c r="H29" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="B30" t="s">
+        <v>129</v>
+      </c>
+      <c r="C30" t="s">
+        <v>130</v>
+      </c>
+      <c r="D30" t="s">
+        <v>11</v>
+      </c>
+      <c r="E30" t="s">
+        <v>103</v>
+      </c>
+      <c r="F30" t="s">
         <v>131</v>
       </c>
-      <c r="C30" t="s">
+      <c r="G30" t="s">
         <v>132</v>
       </c>
-      <c r="D30" t="s">
-        <v>18</v>
-      </c>
-      <c r="E30" t="s">
-        <v>96</v>
-      </c>
-      <c r="F30" t="s">
-        <v>124</v>
-      </c>
-      <c r="G30" t="s">
+      <c r="H30" t="s">
         <v>133</v>
-      </c>
-      <c r="H30" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="B31" t="s">
+        <v>134</v>
+      </c>
+      <c r="C31" t="s">
         <v>135</v>
       </c>
-      <c r="C31" t="s">
+      <c r="D31" t="s">
+        <v>18</v>
+      </c>
+      <c r="E31" t="s">
+        <v>103</v>
+      </c>
+      <c r="F31" t="s">
+        <v>131</v>
+      </c>
+      <c r="G31" t="s">
         <v>136</v>
       </c>
-      <c r="D31" t="s">
-        <v>23</v>
-      </c>
-      <c r="E31" t="s">
-        <v>96</v>
-      </c>
-      <c r="F31" t="s">
-        <v>124</v>
-      </c>
-      <c r="G31" t="s">
+      <c r="H31" t="s">
         <v>137</v>
-      </c>
-      <c r="H31" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="B32" t="s">
-        <v>122</v>
+        <v>138</v>
       </c>
       <c r="C32" t="s">
         <v>139</v>
       </c>
       <c r="D32" t="s">
-        <v>59</v>
+        <v>23</v>
       </c>
       <c r="E32" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="F32" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="G32" t="s">
         <v>140</v>
@@ -1389,94 +1434,94 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
+        <v>128</v>
+      </c>
+      <c r="B33" t="s">
         <v>142</v>
       </c>
-      <c r="B33" t="s">
+      <c r="C33" t="s">
         <v>143</v>
       </c>
-      <c r="C33" t="s">
+      <c r="D33" t="s">
+        <v>28</v>
+      </c>
+      <c r="E33" t="s">
+        <v>103</v>
+      </c>
+      <c r="F33" t="s">
+        <v>131</v>
+      </c>
+      <c r="G33" t="s">
         <v>144</v>
       </c>
-      <c r="D33" t="s">
-        <v>38</v>
-      </c>
-      <c r="E33" t="s">
-        <v>12</v>
-      </c>
-      <c r="F33" t="s">
-        <v>13</v>
-      </c>
-      <c r="G33" t="s">
+      <c r="H33" t="s">
         <v>145</v>
-      </c>
-      <c r="H33" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>142</v>
+        <v>128</v>
       </c>
       <c r="B34" t="s">
+        <v>146</v>
+      </c>
+      <c r="C34" t="s">
         <v>147</v>
       </c>
-      <c r="C34" t="s">
+      <c r="D34" t="s">
+        <v>33</v>
+      </c>
+      <c r="E34" t="s">
+        <v>103</v>
+      </c>
+      <c r="F34" t="s">
+        <v>131</v>
+      </c>
+      <c r="G34" t="s">
         <v>148</v>
       </c>
-      <c r="D34" t="s">
-        <v>11</v>
-      </c>
-      <c r="E34" t="s">
-        <v>12</v>
-      </c>
-      <c r="F34" t="s">
-        <v>13</v>
-      </c>
-      <c r="G34" t="s">
+      <c r="H34" t="s">
         <v>149</v>
-      </c>
-      <c r="H34" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>142</v>
+        <v>128</v>
       </c>
       <c r="B35" t="s">
+        <v>129</v>
+      </c>
+      <c r="C35" t="s">
+        <v>150</v>
+      </c>
+      <c r="D35" t="s">
+        <v>37</v>
+      </c>
+      <c r="E35" t="s">
+        <v>103</v>
+      </c>
+      <c r="F35" t="s">
+        <v>131</v>
+      </c>
+      <c r="G35" t="s">
         <v>151</v>
       </c>
-      <c r="C35" t="s">
+      <c r="H35" t="s">
         <v>152</v>
-      </c>
-      <c r="D35" t="s">
-        <v>18</v>
-      </c>
-      <c r="E35" t="s">
-        <v>12</v>
-      </c>
-      <c r="F35" t="s">
-        <v>13</v>
-      </c>
-      <c r="G35" t="s">
-        <v>153</v>
-      </c>
-      <c r="H35" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>142</v>
+        <v>153</v>
       </c>
       <c r="B36" t="s">
+        <v>154</v>
+      </c>
+      <c r="C36" t="s">
         <v>155</v>
       </c>
-      <c r="C36" t="s">
-        <v>156</v>
-      </c>
       <c r="D36" t="s">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="E36" t="s">
         <v>12</v>
@@ -1485,24 +1530,24 @@
         <v>13</v>
       </c>
       <c r="G36" t="s">
+        <v>156</v>
+      </c>
+      <c r="H36" t="s">
         <v>157</v>
-      </c>
-      <c r="H36" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>142</v>
+        <v>153</v>
       </c>
       <c r="B37" t="s">
-        <v>143</v>
+        <v>158</v>
       </c>
       <c r="C37" t="s">
         <v>159</v>
       </c>
       <c r="D37" t="s">
-        <v>59</v>
+        <v>18</v>
       </c>
       <c r="E37" t="s">
         <v>12</v>
@@ -1515,6 +1560,110 @@
       </c>
       <c r="H37" t="s">
         <v>161</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s">
+        <v>153</v>
+      </c>
+      <c r="B38" t="s">
+        <v>162</v>
+      </c>
+      <c r="C38" t="s">
+        <v>163</v>
+      </c>
+      <c r="D38" t="s">
+        <v>23</v>
+      </c>
+      <c r="E38" t="s">
+        <v>12</v>
+      </c>
+      <c r="F38" t="s">
+        <v>13</v>
+      </c>
+      <c r="G38" t="s">
+        <v>164</v>
+      </c>
+      <c r="H38" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s">
+        <v>153</v>
+      </c>
+      <c r="B39" t="s">
+        <v>166</v>
+      </c>
+      <c r="C39" t="s">
+        <v>167</v>
+      </c>
+      <c r="D39" t="s">
+        <v>28</v>
+      </c>
+      <c r="E39" t="s">
+        <v>12</v>
+      </c>
+      <c r="F39" t="s">
+        <v>13</v>
+      </c>
+      <c r="G39" t="s">
+        <v>168</v>
+      </c>
+      <c r="H39" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s">
+        <v>153</v>
+      </c>
+      <c r="B40" t="s">
+        <v>170</v>
+      </c>
+      <c r="C40" t="s">
+        <v>171</v>
+      </c>
+      <c r="D40" t="s">
+        <v>33</v>
+      </c>
+      <c r="E40" t="s">
+        <v>12</v>
+      </c>
+      <c r="F40" t="s">
+        <v>13</v>
+      </c>
+      <c r="G40" t="s">
+        <v>172</v>
+      </c>
+      <c r="H40" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s">
+        <v>153</v>
+      </c>
+      <c r="B41" t="s">
+        <v>154</v>
+      </c>
+      <c r="C41" t="s">
+        <v>174</v>
+      </c>
+      <c r="D41" t="s">
+        <v>37</v>
+      </c>
+      <c r="E41" t="s">
+        <v>12</v>
+      </c>
+      <c r="F41" t="s">
+        <v>13</v>
+      </c>
+      <c r="G41" t="s">
+        <v>175</v>
+      </c>
+      <c r="H41" t="s">
+        <v>176</v>
       </c>
     </row>
   </sheetData>

</xml_diff>